<commit_message>
Updated RF Board BOM
Updated RF Board BOM
</commit_message>
<xml_diff>
--- a/T41_V012_Files/T41_V012_BOMs/Source Files/T41_RF_Board_BOM_V012.8_09-12-26.xlsx
+++ b/T41_V012_Files/T41_V012_BOMs/Source Files/T41_RF_Board_BOM_V012.8_09-12-26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bill\Documents\GitHub\T41\T41_V012_Files\T41_V012_BOMs\Source Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC76E2EF-3B86-4C11-9FDF-6598C912A942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6EBC54-A64D-4A8C-A9E8-31120366E9FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="743" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -933,7 +933,7 @@
     <t>R7, R9, R12, R15, R19, R20, R21, R23</t>
   </si>
   <si>
-    <t>C37, C54</t>
+    <t>C4, C10, C17, C28, C37, C54</t>
   </si>
 </sst>
 </file>
@@ -1565,7 +1565,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B6" t="s">
         <v>287</v>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="H6" s="5">
         <f t="shared" si="0"/>
-        <v>0.22</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -3056,14 +3056,14 @@
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A55" s="1">
         <f>SUM(A2:A54)</f>
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D55" t="s">
         <v>54</v>
       </c>
       <c r="H55" s="10">
         <f>SUM(H2:H54)</f>
-        <v>92.921000000000006</v>
+        <v>93.361000000000004</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">

</xml_diff>